<commit_message>
This is a large commit. I got carried away and completed and updated the following in one big commit. Added figures for carrots, mesclun, and tomatoes. Added a markdown file for perfect competition analysis. Updated the marginal analysis readme and model. Deleted the old memo template and added a new memo for perfect competition. Updated the prompt log.
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alaskaair-my.sharepoint.com/personal/wade_okumura_alaskaair_com/Documents/Documents/EMBA/2026 Fall/Bus 620 - Econ/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alaskaair-my.sharepoint.com/personal/wade_okumura_alaskaair_com/Documents/Documents/GitHub/wade-okumura/capabilities/marginal-analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E7D35FC-A469-436C-95BE-8B81D7D3A2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{1E7D35FC-A469-436C-95BE-8B81D7D3A2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C363FDBC-1CC2-45A5-A075-F5511B85F8E3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -1265,11 +1265,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2146,17 +2146,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2970,17 +2970,17 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B25" s="31"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -3794,17 +3794,17 @@
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="31" t="s">
+      <c r="A49" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="B49" s="31"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="31"/>
-      <c r="E49" s="31"/>
-      <c r="F49" s="31"/>
-      <c r="G49" s="31"/>
-      <c r="H49" s="31"/>
-      <c r="I49" s="31"/>
+      <c r="B49" s="30"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="30"/>
+      <c r="E49" s="30"/>
+      <c r="F49" s="30"/>
+      <c r="G49" s="30"/>
+      <c r="H49" s="30"/>
+      <c r="I49" s="30"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
@@ -5001,10 +5001,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="30"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -5057,10 +5057,10 @@
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="31"/>
+      <c r="B7" s="30"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -5237,13 +5237,13 @@
       <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
@@ -5508,134 +5508,134 @@
       <c r="E37" s="1"/>
     </row>
     <row r="38" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="30"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B39" s="30" t="s">
+      <c r="B39" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="30"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B40" s="30" t="s">
+      <c r="B40" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="30"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B41" s="30" t="s">
+      <c r="B41" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
-      <c r="E41" s="30"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B42" s="30" t="s">
+      <c r="B42" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="30"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="31"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B43" s="30" t="s">
+      <c r="B43" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="31"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B45" s="30" t="s">
+      <c r="B45" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B46" s="30" t="s">
+      <c r="B46" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="31"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B47" s="30" t="s">
+      <c r="B47" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B48" s="30" t="s">
+      <c r="B48" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="31"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B49" s="30" t="s">
+      <c r="B49" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="30"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="31"/>
+      <c r="E49" s="31"/>
     </row>
   </sheetData>
   <scenarios current="0">
@@ -5646,21 +5646,21 @@
     </scenario>
   </scenarios>
   <mergeCells count="15">
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B44:E44"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B49:E49"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" sqref="B21" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -5954,12 +5954,12 @@
       <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">

</xml_diff>